<commit_message>
Epic 1 Close-out: Alpha QA Pass & Findings Memo (Task #81)
- All regression tests pass: 115 golden-model assertions, 24 exports
- Frontend builds clean (vite build succeeds)
- E2E tests pass: login, wizard flow, consultant analysis, KPI drawers
- Updated docs/epic1-findings.md with corrected facts:
  - 13 explainers (not 14)
  - 10 coaching event types (not 11)
  - Server-side guidance-level validation now exists (risk #4 resolved)
  - Frontend typecheck has 19 type errors (type definition gaps, not runtime)
  - Added E2E coverage section and event tracking verification
</commit_message>
<xml_diff>
--- a/artifacts/api-server/qa-output/Underwriting_V2_(21-tab)_Charter_ADA_Grade-Band.xlsx
+++ b/artifacts/api-server/qa-output/Underwriting_V2_(21-tab)_Charter_ADA_Grade-Band.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="702" uniqueCount="378">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="702" uniqueCount="379">
   <si>
     <t>SchoolStack Budget</t>
   </si>
@@ -504,10 +504,13 @@
     <t>Salary Escalation Rate</t>
   </si>
   <si>
-    <t>Derived from tuition escalation rate</t>
+    <t>Salary input or tuition escalation fallback</t>
   </si>
   <si>
     <t>Cost Inflation Rate</t>
+  </si>
+  <si>
+    <t>Cost inflation input or tuition escalation fallback</t>
   </si>
   <si>
     <t>Year 1 Proration Factor</t>
@@ -2057,7 +2060,7 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="11" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B1" s="11"/>
       <c r="C1" s="11"/>
@@ -2107,7 +2110,7 @@
     </row>
     <row r="6" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="13" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B6" s="13"/>
       <c r="C6" s="13"/>
@@ -2237,7 +2240,7 @@
     </row>
     <row r="13" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="13" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B13" s="27">
         <f>SUM(B7:B12)</f>
@@ -2262,7 +2265,7 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B15" s="26">
         <v>11783</v>
@@ -2306,7 +2309,7 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="11" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B1" s="11"/>
       <c r="C1" s="11"/>
@@ -2346,7 +2349,7 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B5" s="26">
         <v>278438</v>
@@ -2366,7 +2369,7 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B6" s="26">
         <v>59029</v>
@@ -2386,7 +2389,7 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="B7" s="26">
         <v>87955</v>
@@ -2406,7 +2409,7 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="B8" s="31">
         <f>SUM(B5:B7)</f>
@@ -2441,7 +2444,7 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="B10" s="26">
         <v>116944</v>
@@ -2461,7 +2464,7 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B11" s="26">
         <v>91328</v>
@@ -2481,7 +2484,7 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="B12" s="31">
         <f>SUM(B10:B11)</f>
@@ -2516,7 +2519,7 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="B14" s="26">
         <v>69053</v>
@@ -2536,7 +2539,7 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="B15" s="31">
         <f>SUM(B14:B14)</f>
@@ -2571,7 +2574,7 @@
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="B17" s="26">
         <v>77790</v>
@@ -2591,7 +2594,7 @@
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="B18" s="31">
         <f>SUM(B17:B17)</f>
@@ -2616,7 +2619,7 @@
     </row>
     <row r="20" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="13" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="B20" s="27">
         <f>B8+B12+B15+B18</f>
@@ -2665,7 +2668,7 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="11" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="B1" s="11"/>
       <c r="C1" s="11"/>
@@ -2695,7 +2698,7 @@
     </row>
     <row r="4" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="13" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="B4" s="13"/>
       <c r="C4" s="13"/>
@@ -2705,7 +2708,7 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="B5" s="26">
         <v>807500</v>
@@ -2725,7 +2728,7 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="B6" s="26">
         <v>75000</v>
@@ -2745,7 +2748,7 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="B7" s="26">
         <v>110000</v>
@@ -2765,7 +2768,7 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="B8" s="26">
         <v>125000</v>
@@ -2785,7 +2788,7 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B9" s="26">
         <v>20833</v>
@@ -2805,7 +2808,7 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="B10" s="26">
         <v>40000</v>
@@ -2825,7 +2828,7 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="B11" s="31">
         <f>SUM(B5:B10)</f>
@@ -2850,7 +2853,7 @@
     </row>
     <row r="13" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="13" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="B13" s="13"/>
       <c r="C13" s="13"/>
@@ -2860,7 +2863,7 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="B14" s="26">
         <v>116944</v>
@@ -2880,7 +2883,7 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B15" s="26">
         <v>91328</v>
@@ -2900,7 +2903,7 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B16" s="26">
         <v>278438</v>
@@ -2920,7 +2923,7 @@
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B17" s="26">
         <v>59029</v>
@@ -2940,7 +2943,7 @@
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="B18" s="26">
         <v>87955</v>
@@ -2960,7 +2963,7 @@
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="B19" s="26">
         <v>69053</v>
@@ -2980,7 +2983,7 @@
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="B20" s="26">
         <v>77790</v>
@@ -3000,7 +3003,7 @@
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B21" s="31">
         <f>SUM(B14:B20)</f>
@@ -3040,7 +3043,7 @@
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="4" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="B25" s="26">
         <v>65000</v>
@@ -3065,7 +3068,7 @@
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="4" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="B27" s="26">
         <v>45000</v>
@@ -3090,7 +3093,7 @@
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="4" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="B29" s="26">
         <v>220000</v>
@@ -3110,7 +3113,7 @@
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="B30" s="26">
         <v>30000</v>
@@ -3130,7 +3133,7 @@
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="4" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="B31" s="26">
         <v>18333</v>
@@ -3150,7 +3153,7 @@
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="B32" s="31">
         <f>SUM(B29:B31)</f>
@@ -3180,7 +3183,7 @@
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" s="4" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="B34" s="26">
         <v>25000</v>
@@ -3200,7 +3203,7 @@
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" s="4" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="B35" s="26">
         <v>10000</v>
@@ -3220,7 +3223,7 @@
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" s="4" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="B36" s="26">
         <v>15000</v>
@@ -3240,7 +3243,7 @@
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" s="4" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="B37" s="26">
         <v>75000</v>
@@ -3260,7 +3263,7 @@
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" s="3" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="B38" s="31">
         <f>SUM(B34:B37)</f>
@@ -3285,7 +3288,7 @@
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" s="3" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="B39" s="31">
         <f>B25+B27+B32+B38</f>
@@ -3310,7 +3313,7 @@
     </row>
     <row r="41" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" s="13" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="B41" s="13"/>
       <c r="C41" s="13"/>
@@ -3320,7 +3323,7 @@
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" s="4" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="B42" s="26">
         <v>46629</v>
@@ -3340,7 +3343,7 @@
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" s="4" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="B43" s="26">
         <v>60000</v>
@@ -3360,7 +3363,7 @@
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="B44" s="31">
         <f>SUM(B42:B43)</f>
@@ -3409,7 +3412,7 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="11" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="B1" s="11"/>
       <c r="C1" s="11"/>
@@ -3439,7 +3442,7 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="B4" s="29">
         <f>'Budget Detail'!B11</f>
@@ -3464,7 +3467,7 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B5" s="29">
         <f>'Budget Detail'!B21</f>
@@ -3489,7 +3492,7 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="B6" s="29">
         <f>'Budget Detail'!B39</f>
@@ -3514,7 +3517,7 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="B7" s="29">
         <f>'Budget Detail'!B44</f>
@@ -3539,7 +3542,7 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="B8" s="31">
         <f>SUM(B5:B7)</f>
@@ -3564,7 +3567,7 @@
     </row>
     <row r="10" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="13" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="B10" s="13"/>
       <c r="C10" s="13"/>
@@ -3574,7 +3577,7 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B11" s="27">
         <f>B4-B8</f>
@@ -3599,7 +3602,7 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="B12" s="25">
         <f>IF(B4=0,0,B11/B4)</f>
@@ -3624,7 +3627,7 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="B13" s="26">
         <v>-212164</v>
@@ -3644,7 +3647,7 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B14" s="26">
         <v>9819</v>
@@ -3664,7 +3667,7 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="B15" s="26">
         <v>11587</v>
@@ -3709,7 +3712,7 @@
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="11" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="B1" s="11"/>
       <c r="C1" s="11"/>
@@ -3730,48 +3733,48 @@
         <v>67</v>
       </c>
       <c r="B2" s="15" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="C2" s="15" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="D2" s="15" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="E2" s="15" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="F2" s="15" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="G2" s="15" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="H2" s="15" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="I2" s="15" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="J2" s="15" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="K2" s="15" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="L2" s="15" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="M2" s="15" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="N2" s="15" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
     </row>
     <row r="3" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" s="13" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="B3" s="13"/>
       <c r="C3" s="13"/>
@@ -3789,7 +3792,7 @@
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="B4" s="31">
         <v>146500</v>
@@ -3833,7 +3836,7 @@
     </row>
     <row r="6" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" s="13" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="B6" s="13"/>
       <c r="C6" s="13"/>
@@ -3851,7 +3854,7 @@
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="B7" s="26">
         <v>78054</v>
@@ -3895,7 +3898,7 @@
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="B8" s="26">
         <v>50333</v>
@@ -3939,7 +3942,7 @@
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="B9" s="26">
         <v>8886</v>
@@ -3983,7 +3986,7 @@
     </row>
     <row r="11" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" s="13" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="B11" s="13"/>
       <c r="C11" s="13"/>
@@ -4001,7 +4004,7 @@
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="B12" s="29">
         <v>137273</v>
@@ -4045,7 +4048,7 @@
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="B13" s="29">
         <v>9227</v>
@@ -4089,7 +4092,7 @@
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="B14" s="34">
         <v>9227</v>
@@ -4133,14 +4136,14 @@
     </row>
     <row r="16" ht="24" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="13" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="B16" s="13"/>
       <c r="C16" s="13"/>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B17" s="26">
         <v>0</v>
@@ -4148,7 +4151,7 @@
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="B18" s="34">
         <v>74498</v>
@@ -4156,7 +4159,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="B19" s="26">
         <v>9227</v>
@@ -4188,7 +4191,7 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="11" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="B1" s="11"/>
       <c r="C1" s="11"/>
@@ -4218,7 +4221,7 @@
     </row>
     <row r="4" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="13" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="B4" s="13"/>
       <c r="C4" s="13"/>
@@ -4228,7 +4231,7 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="35" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="B5" s="31">
         <v>1178333</v>
@@ -4248,7 +4251,7 @@
     </row>
     <row r="7" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="13" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="B7" s="13"/>
       <c r="C7" s="13"/>
@@ -4258,7 +4261,7 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="B8" s="29">
         <v>780535</v>
@@ -4278,7 +4281,7 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="B9" s="29">
         <v>503333</v>
@@ -4298,7 +4301,7 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="B10" s="29">
         <v>106629</v>
@@ -4318,7 +4321,7 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="35" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="B11" s="31">
         <f>SUM(B8:B10)</f>
@@ -4343,7 +4346,7 @@
     </row>
     <row r="13" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="13" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="B13" s="13"/>
       <c r="C13" s="13"/>
@@ -4353,7 +4356,7 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="35" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B14" s="27">
         <f>B5-B11</f>
@@ -4378,7 +4381,7 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="B15" s="25">
         <f>IF(B5=0,0,B14/B5)</f>
@@ -4467,7 +4470,7 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="B5" s="26">
         <v>350000</v>
@@ -4487,7 +4490,7 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="B6" s="26">
         <v>20283</v>
@@ -4507,7 +4510,7 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="B7" s="26">
         <v>26345</v>
@@ -4527,7 +4530,7 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="B8" s="29">
         <v>46629</v>
@@ -4547,7 +4550,7 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="B9" s="34">
         <v>323655</v>
@@ -4591,7 +4594,7 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="11" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="B1" s="11"/>
       <c r="C1" s="11"/>
@@ -4621,7 +4624,7 @@
     </row>
     <row r="4" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="13" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="B4" s="13"/>
       <c r="C4" s="13"/>
@@ -4631,7 +4634,7 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="B5" s="36">
         <v>74498</v>
@@ -4651,7 +4654,7 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B6" s="26">
         <v>0</v>
@@ -4671,7 +4674,7 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="B7" s="26">
         <v>0</v>
@@ -4691,7 +4694,7 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="B8" s="26">
         <v>0</v>
@@ -4711,7 +4714,7 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="B9" s="31">
         <v>74498</v>
@@ -4731,7 +4734,7 @@
     </row>
     <row r="11" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="13" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="B11" s="13"/>
       <c r="C11" s="13"/>
@@ -4741,7 +4744,7 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="B12" s="26">
         <v>0</v>
@@ -4761,7 +4764,7 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="B13" s="26">
         <v>323655</v>
@@ -4781,7 +4784,7 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="B14" s="31">
         <v>323655</v>
@@ -4801,7 +4804,7 @@
     </row>
     <row r="16" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="13" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="B16" s="13"/>
       <c r="C16" s="13"/>
@@ -4811,7 +4814,7 @@
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="B17" s="27">
         <v>-249157</v>
@@ -4831,7 +4834,7 @@
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="B19" s="37">
         <v>0</v>
@@ -4875,7 +4878,7 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="11" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="B1" s="11"/>
       <c r="C1" s="11"/>
@@ -4905,7 +4908,7 @@
     </row>
     <row r="4" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="13" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="B4" s="13"/>
       <c r="C4" s="13"/>
@@ -4915,7 +4918,7 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="B5" s="26">
         <v>1178333</v>
@@ -4935,7 +4938,7 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="B6" s="26">
         <v>780535</v>
@@ -4955,7 +4958,7 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="B7" s="26">
         <v>503333</v>
@@ -4975,7 +4978,7 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="B8" s="29">
         <f>B5-B6-B7</f>
@@ -5000,7 +5003,7 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="B9" s="26">
         <v>46629</v>
@@ -5020,7 +5023,7 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="B10" s="39">
         <f>IF(B9=0,"N/A",B8/B9)</f>
@@ -5045,7 +5048,7 @@
     </row>
     <row r="12" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="13" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="B12" s="13"/>
       <c r="C12" s="13"/>
@@ -5055,7 +5058,7 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="B13" s="26">
         <v>74498</v>
@@ -5075,7 +5078,7 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="B14" s="23">
         <f>IF((B6+B7+B9)=0,0,(B13/(B6+B7+B9))*365)</f>
@@ -5100,7 +5103,7 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="B15" s="30">
         <f>IF((B6+B7+B9)=0,0,B13/((B6+B7+B9)/12))</f>
@@ -5125,7 +5128,7 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B16" s="25">
         <v>0.2</v>
@@ -5145,7 +5148,7 @@
     </row>
     <row r="18" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="13" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="B18" s="13"/>
       <c r="C18" s="13"/>
@@ -5155,7 +5158,7 @@
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B19" s="26">
         <v>9819</v>
@@ -5175,7 +5178,7 @@
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="B20" s="26">
         <v>827164</v>
@@ -5195,7 +5198,7 @@
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="B21" s="26">
         <v>4194</v>
@@ -5215,7 +5218,7 @@
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="B22" s="40">
         <v>148</v>
@@ -5235,7 +5238,7 @@
     </row>
     <row r="24" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="13" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="B24" s="13"/>
       <c r="C24" s="13"/>
@@ -5245,102 +5248,102 @@
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="4" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="B25" s="41" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="C25" s="42" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="D25" s="42" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="E25" s="42" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="F25" s="42" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
+        <v>349</v>
+      </c>
+      <c r="B26" s="41" t="s">
+        <v>347</v>
+      </c>
+      <c r="C26" s="42" t="s">
         <v>348</v>
       </c>
-      <c r="B26" s="41" t="s">
-        <v>346</v>
-      </c>
-      <c r="C26" s="42" t="s">
-        <v>347</v>
-      </c>
       <c r="D26" s="42" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="E26" s="42" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="F26" s="42" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="4" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="B27" s="41" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="C27" s="41" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="D27" s="41" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="E27" s="41" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="F27" s="41" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="4" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="B28" s="41" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="C28" s="42" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="D28" s="42" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="E28" s="42" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="F28" s="42" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="4" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="B29" s="41" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="C29" s="42" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="D29" s="42" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="E29" s="42" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="F29" s="42" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
     </row>
   </sheetData>
@@ -5381,13 +5384,13 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="43" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="B3" s="43" t="s">
         <v>100</v>
       </c>
       <c r="D3" s="43" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="E3" s="43" t="s">
         <v>100</v>
@@ -5401,7 +5404,7 @@
         <v>350000</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="E4" s="26">
         <v>250000</v>
@@ -5409,7 +5412,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="B5" s="26">
         <v>150000</v>
@@ -5423,7 +5426,7 @@
     </row>
     <row r="6" spans="4:5" x14ac:dyDescent="0.25">
       <c r="D6" s="4" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="E6" s="26">
         <v>50000</v>
@@ -5431,7 +5434,7 @@
     </row>
     <row r="7" spans="4:5" x14ac:dyDescent="0.25">
       <c r="D7" s="4" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="E7" s="26">
         <v>140000</v>
@@ -5439,13 +5442,13 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="B9" s="27">
         <v>500000</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="E9" s="27">
         <v>500000</v>
@@ -5453,7 +5456,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="B10" s="37">
         <v>0</v>
@@ -5621,7 +5624,7 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="11" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="B1" s="11"/>
       <c r="C1" s="11"/>
@@ -5631,7 +5634,7 @@
     </row>
     <row r="3" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="13" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="B3" s="13"/>
       <c r="C3" s="13"/>
@@ -5641,7 +5644,7 @@
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
     </row>
     <row r="5" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -5666,7 +5669,7 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="B6" s="26">
         <v>1178333</v>
@@ -5686,7 +5689,7 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="B7" s="26">
         <v>1330497</v>
@@ -5706,7 +5709,7 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B8" s="27">
         <v>-152164</v>
@@ -5726,7 +5729,7 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="B9" s="25">
         <v>-0.12913460606689658</v>
@@ -5746,7 +5749,7 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="B10" s="44">
         <v>-2.26</v>
@@ -5766,7 +5769,7 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="B11" s="23">
         <v>148</v>
@@ -5786,7 +5789,7 @@
     </row>
     <row r="13" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="13" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="B13" s="13"/>
       <c r="C13" s="13"/>
@@ -5796,7 +5799,7 @@
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" s="12" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
     </row>
     <row r="15" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -5821,7 +5824,7 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="B16" s="26">
         <v>1001583</v>
@@ -5841,7 +5844,7 @@
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="B17" s="26">
         <v>1330497</v>
@@ -5861,7 +5864,7 @@
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B18" s="27">
         <v>-328914</v>
@@ -5881,7 +5884,7 @@
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="B19" s="25">
         <v>-0.32839365419634886</v>
@@ -5901,7 +5904,7 @@
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="B20" s="44">
         <v>-6.05</v>
@@ -5921,7 +5924,7 @@
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="B21" s="23">
         <v>170</v>
@@ -5941,7 +5944,7 @@
     </row>
     <row r="23" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="13" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="B23" s="13"/>
       <c r="C23" s="13"/>
@@ -5951,7 +5954,7 @@
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" s="12" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
     </row>
     <row r="25" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -5976,7 +5979,7 @@
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="B26" s="26">
         <v>1084067</v>
@@ -5996,7 +5999,7 @@
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="4" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="B27" s="26">
         <v>1330497</v>
@@ -6016,7 +6019,7 @@
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B28" s="27">
         <v>-246430</v>
@@ -6036,7 +6039,7 @@
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="4" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="B29" s="25">
         <v>-0.2273202239857572</v>
@@ -6056,7 +6059,7 @@
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="B30" s="44">
         <v>-4.28</v>
@@ -6076,7 +6079,7 @@
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="4" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="B31" s="23">
         <v>171</v>
@@ -6122,7 +6125,7 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="11" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="B1" s="11"/>
       <c r="C1" s="11"/>
@@ -6156,7 +6159,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>7</v>
@@ -6180,7 +6183,7 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>17</v>
@@ -6188,7 +6191,7 @@
     </row>
     <row r="11" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="13" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="B11" s="13"/>
       <c r="C11" s="13"/>
@@ -6226,7 +6229,7 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="D13" s="26">
         <v>1178333</v>
@@ -6246,7 +6249,7 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D14" s="26">
         <v>1330497</v>
@@ -6266,7 +6269,7 @@
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="D15" s="26">
         <v>-212164</v>
@@ -6286,7 +6289,7 @@
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="D16" s="26">
         <v>74498</v>
@@ -6306,7 +6309,7 @@
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="D17" s="26">
         <v>323655</v>
@@ -6326,7 +6329,7 @@
     </row>
     <row r="19" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" s="13" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="B19" s="13"/>
       <c r="C19" s="13"/>
@@ -6364,7 +6367,7 @@
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="D21" s="25">
         <v>-0.18005398371894768</v>
@@ -6384,7 +6387,7 @@
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" s="4" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="D22" s="44">
         <v>-2.26</v>
@@ -6404,7 +6407,7 @@
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" s="4" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="D23" s="25">
         <v>0.2</v>
@@ -6424,7 +6427,7 @@
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="D24" s="23">
         <v>120</v>
@@ -6444,7 +6447,7 @@
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" s="8" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="8"/>
@@ -7228,12 +7231,12 @@
         <v>0.03</v>
       </c>
       <c r="C57" s="20" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A58" s="4" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B58" s="19">
         <v>0.8333333333333334</v>
@@ -7241,7 +7244,7 @@
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A59" s="4" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B59" s="17">
         <v>0</v>
@@ -7249,15 +7252,15 @@
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A60" s="4" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B60" s="14" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="62" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="13" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B62" s="13"/>
       <c r="C62" s="13"/>
@@ -7268,15 +7271,15 @@
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A63" s="4" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B63" s="14" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A64" s="4" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B64" s="14" t="s">
         <v>135</v>
@@ -7284,7 +7287,7 @@
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A65" s="4" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B65" s="16">
         <v>0</v>
@@ -7292,7 +7295,7 @@
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A66" s="4" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B66" s="16">
         <v>0</v>
@@ -7300,7 +7303,7 @@
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A67" s="4" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B67" s="21">
         <v>0.95</v>
@@ -7308,21 +7311,21 @@
     </row>
     <row r="69" ht="28" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" s="15" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B69" s="15" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C69" s="15" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D69" s="15" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70" s="4" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B70" s="17">
         <v>8200</v>
@@ -7336,7 +7339,7 @@
     </row>
     <row r="72" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72" s="15" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B72" s="15" t="s">
         <v>90</v>
@@ -7356,7 +7359,7 @@
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73" s="4" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B73" s="16">
         <v>80</v>
@@ -7376,7 +7379,7 @@
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74" s="4" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B74" s="16">
         <v>40</v>
@@ -7396,7 +7399,7 @@
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A75" s="4" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B75" s="16">
         <v>0</v>
@@ -7446,10 +7449,10 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -7470,10 +7473,10 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -7486,7 +7489,7 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B8" s="4" t="s">
         <v>17</v>
@@ -7497,31 +7500,31 @@
         <v>87</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
@@ -7529,31 +7532,31 @@
         <v>88</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
   </sheetData>
@@ -7613,7 +7616,7 @@
     </row>
     <row r="5" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="13" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B5" s="13"/>
       <c r="C5" s="13"/>
@@ -7651,7 +7654,7 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B8" s="24">
         <v>0.2</v>
@@ -7671,10 +7674,10 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="C10" s="25">
         <v>0.6666666666666666</v>
@@ -7715,7 +7718,7 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="11" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="B1" s="11"/>
       <c r="C1" s="11"/>
@@ -7745,7 +7748,7 @@
     </row>
     <row r="4" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="13" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B4" s="13"/>
       <c r="C4" s="13"/>
@@ -7755,7 +7758,7 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B5" s="26">
         <v>969000</v>
@@ -7775,7 +7778,7 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B6" s="26">
         <v>90000</v>
@@ -7795,7 +7798,7 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B7" s="26">
         <v>132000</v>
@@ -7815,7 +7818,7 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B8" s="26">
         <v>150000</v>
@@ -7835,7 +7838,7 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B9" s="26">
         <v>25000</v>
@@ -7855,7 +7858,7 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B10" s="26">
         <v>48000</v>
@@ -7875,7 +7878,7 @@
     </row>
     <row r="11" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="13" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B11" s="27">
         <f>SUM(B5:B10)</f>
@@ -7948,7 +7951,7 @@
         <v>116</v>
       </c>
       <c r="D3" s="15" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="E3" s="15" t="s">
         <v>118</v>
@@ -7957,7 +7960,7 @@
         <v>119</v>
       </c>
       <c r="G3" s="15" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -8123,7 +8126,7 @@
     </row>
     <row r="12" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="13" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B12" s="13"/>
       <c r="C12" s="13"/>
@@ -8154,7 +8157,7 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B14" s="27">
         <v>780535</v>
@@ -8174,7 +8177,7 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B15" s="25">
         <v>0.5520049504950495</v>
@@ -8194,7 +8197,7 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="B16" s="30">
         <v>8.6</v>
@@ -8238,7 +8241,7 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="11" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B1" s="11"/>
       <c r="C1" s="11"/>
@@ -8278,7 +8281,7 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B5" s="26">
         <v>78000</v>
@@ -8298,7 +8301,7 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="B6" s="31">
         <f>SUM(B5:B5)</f>
@@ -8333,7 +8336,7 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="B8" s="26">
         <v>54000</v>
@@ -8353,7 +8356,7 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="B9" s="31">
         <f>SUM(B8:B8)</f>
@@ -8388,7 +8391,7 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B11" s="26">
         <v>264000</v>
@@ -8408,7 +8411,7 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="B12" s="26">
         <v>36000</v>
@@ -8428,7 +8431,7 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B13" s="26">
         <v>22000</v>
@@ -8448,7 +8451,7 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B14" s="31">
         <f>SUM(B11:B13)</f>
@@ -8483,7 +8486,7 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B16" s="26">
         <v>30000</v>
@@ -8503,7 +8506,7 @@
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B17" s="26">
         <v>12000</v>
@@ -8523,7 +8526,7 @@
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B18" s="26">
         <v>18000</v>
@@ -8543,7 +8546,7 @@
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B19" s="26">
         <v>90000</v>
@@ -8563,7 +8566,7 @@
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="B20" s="31">
         <f>SUM(B16:B19)</f>
@@ -8588,7 +8591,7 @@
     </row>
     <row r="22" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="13" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B22" s="27">
         <f>B6+B9+B14+B20</f>
@@ -8638,7 +8641,7 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="11" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B1" s="11"/>
       <c r="C1" s="11"/>
@@ -8663,7 +8666,7 @@
         <v>150</v>
       </c>
       <c r="F3" s="15" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -8691,7 +8694,7 @@
         <v>153</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C5" s="17">
         <v>60000</v>
@@ -8708,7 +8711,7 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="F7" s="27">
         <v>46629</v>
@@ -8716,7 +8719,7 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="F8" s="31">
         <v>350000</v>

</xml_diff>

<commit_message>
Add formulas to calculate monthly cash flow and total expenses
Updates the `underwriting-workbook.ts` file to implement formulas for total revenue, personnel, operating expenses, debt service, total expenses, net cash flow, and cumulative cash flow within the Monthly Cash Flow Y1 section. Also updates QA report file sizes.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: a1e7a024-8deb-4e05-bb93-350fde674463
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: e7f3deba-c69f-4f57-99dc-70e82ba15edc
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/27fdbaf7-67db-442f-83d4-bebcb570d0b5/a1e7a024-8deb-4e05-bb93-350fde674463/elh1MDR
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/artifacts/api-server/qa-output/Underwriting_V2_(21-tab)_Charter_ADA_Grade-Band.xlsx
+++ b/artifacts/api-server/qa-output/Underwriting_V2_(21-tab)_Charter_ADA_Grade-Band.xlsx
@@ -3867,6 +3867,7 @@
         <v>0</v>
       </c>
       <c r="N4" s="31">
+        <f>SUM(B4:M4)</f>
         <v>1465000</v>
       </c>
     </row>
@@ -3929,6 +3930,7 @@
         <v>0</v>
       </c>
       <c r="N7" s="26">
+        <f>SUM(B7:M7)</f>
         <v>780535</v>
       </c>
     </row>
@@ -3973,6 +3975,7 @@
         <v>0</v>
       </c>
       <c r="N8" s="26">
+        <f>SUM(B8:M8)</f>
         <v>503333</v>
       </c>
     </row>
@@ -4017,6 +4020,7 @@
         <v>8886</v>
       </c>
       <c r="N9" s="26">
+        <f>SUM(B9:M9)</f>
         <v>106629</v>
       </c>
     </row>
@@ -4043,42 +4047,55 @@
         <v>286</v>
       </c>
       <c r="B12" s="29">
+        <f>B7+B8+B9</f>
         <v>137273</v>
       </c>
       <c r="C12" s="29">
+        <f>C7+C8+C9</f>
         <v>137273</v>
       </c>
       <c r="D12" s="29">
+        <f>D7+D8+D9</f>
         <v>137273</v>
       </c>
       <c r="E12" s="29">
+        <f>E7+E8+E9</f>
         <v>137273</v>
       </c>
       <c r="F12" s="29">
+        <f>F7+F8+F9</f>
         <v>137273</v>
       </c>
       <c r="G12" s="29">
+        <f>G7+G8+G9</f>
         <v>137273</v>
       </c>
       <c r="H12" s="29">
+        <f>H7+H8+H9</f>
         <v>137273</v>
       </c>
       <c r="I12" s="29">
+        <f>I7+I8+I9</f>
         <v>137273</v>
       </c>
       <c r="J12" s="29">
+        <f>J7+J8+J9</f>
         <v>137273</v>
       </c>
       <c r="K12" s="29">
+        <f>K7+K8+K9</f>
         <v>137273</v>
       </c>
       <c r="L12" s="29">
+        <f>L7+L8+L9</f>
         <v>8886</v>
       </c>
       <c r="M12" s="29">
+        <f>M7+M8+M9</f>
         <v>8886</v>
       </c>
       <c r="N12" s="29">
+        <f>SUM(B12:M12)</f>
         <v>1390502</v>
       </c>
     </row>
@@ -4087,42 +4104,55 @@
         <v>311</v>
       </c>
       <c r="B13" s="29">
+        <f>B4-B12</f>
         <v>9227</v>
       </c>
       <c r="C13" s="29">
+        <f>C4-C12</f>
         <v>9227</v>
       </c>
       <c r="D13" s="29">
+        <f>D4-D12</f>
         <v>9227</v>
       </c>
       <c r="E13" s="29">
+        <f>E4-E12</f>
         <v>9227</v>
       </c>
       <c r="F13" s="29">
+        <f>F4-F12</f>
         <v>9227</v>
       </c>
       <c r="G13" s="29">
+        <f>G4-G12</f>
         <v>9227</v>
       </c>
       <c r="H13" s="29">
+        <f>H4-H12</f>
         <v>9227</v>
       </c>
       <c r="I13" s="29">
+        <f>I4-I12</f>
         <v>9227</v>
       </c>
       <c r="J13" s="29">
+        <f>J4-J12</f>
         <v>9227</v>
       </c>
       <c r="K13" s="29">
+        <f>K4-K12</f>
         <v>9227</v>
       </c>
       <c r="L13" s="29">
+        <f>L4-L12</f>
         <v>-8886</v>
       </c>
       <c r="M13" s="29">
+        <f>M4-M12</f>
         <v>-8886</v>
       </c>
       <c r="N13" s="29">
+        <f>SUM(B13:M13)</f>
         <v>74498</v>
       </c>
     </row>
@@ -4131,42 +4161,55 @@
         <v>312</v>
       </c>
       <c r="B14" s="34">
+        <f>B17+B13</f>
         <v>9227</v>
       </c>
       <c r="C14" s="34">
+        <f>B14+C13</f>
         <v>18454</v>
       </c>
       <c r="D14" s="34">
+        <f>C14+D13</f>
         <v>27681</v>
       </c>
       <c r="E14" s="34">
+        <f>D14+E13</f>
         <v>36908</v>
       </c>
       <c r="F14" s="34">
+        <f>E14+F13</f>
         <v>46135</v>
       </c>
       <c r="G14" s="34">
+        <f>F14+G13</f>
         <v>55362</v>
       </c>
       <c r="H14" s="34">
+        <f>G14+H13</f>
         <v>64589</v>
       </c>
       <c r="I14" s="34">
+        <f>H14+I13</f>
         <v>73816</v>
       </c>
       <c r="J14" s="34">
+        <f>I14+J13</f>
         <v>83043</v>
       </c>
       <c r="K14" s="34">
+        <f>J14+K13</f>
         <v>92270</v>
       </c>
       <c r="L14" s="34">
+        <f>K14+L13</f>
         <v>83384</v>
       </c>
       <c r="M14" s="34">
+        <f>L14+M13</f>
         <v>74498</v>
       </c>
       <c r="N14" s="27">
+        <f>M14</f>
         <v>74498</v>
       </c>
     </row>
@@ -4181,7 +4224,7 @@
       <c r="A17" s="4" t="s">
         <v>167</v>
       </c>
-      <c r="B17" s="26">
+      <c r="B17" s="17">
         <v>0</v>
       </c>
     </row>
@@ -4190,6 +4233,7 @@
         <v>314</v>
       </c>
       <c r="B18" s="34">
+        <f>M14</f>
         <v>74498</v>
       </c>
     </row>
@@ -4198,6 +4242,7 @@
         <v>315</v>
       </c>
       <c r="B19" s="26">
+        <f>MIN(B14:M14)</f>
         <v>9227</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update financial statements to include cross-tab references for formulas
Introduces CrossTabRefs interface and updates `buildMonthlyCashFlowY1`, `buildOperatingStatement`, and `buildBalanceSheet` functions in `underwriting-workbook.ts` to support cross-tab references for improved formula calculations. Also updates multiple .xlsx QA output files.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: a1e7a024-8deb-4e05-bb93-350fde674463
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 8084cc2d-73c1-4c39-bbe1-cc56720ed958
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/27fdbaf7-67db-442f-83d4-bebcb570d0b5/a1e7a024-8deb-4e05-bb93-350fde674463/elh1MDR
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/artifacts/api-server/qa-output/Underwriting_V2_(21-tab)_Charter_ADA_Grade-Band.xlsx
+++ b/artifacts/api-server/qa-output/Underwriting_V2_(21-tab)_Charter_ADA_Grade-Band.xlsx
@@ -4788,18 +4788,23 @@
         <v>331</v>
       </c>
       <c r="B5" s="39">
+        <f>'Monthly Cash Flow Y1'!M14</f>
         <v>74498</v>
       </c>
       <c r="C5" s="39">
+        <f>B5+'5-Year Operating Stmt'!C14</f>
         <v>530168</v>
       </c>
       <c r="D5" s="39">
+        <f>B5+'5-Year Operating Stmt'!C14+'5-Year Operating Stmt'!D14</f>
         <v>1838758</v>
       </c>
       <c r="E5" s="39">
+        <f>B5+'5-Year Operating Stmt'!C14+'5-Year Operating Stmt'!D14+'5-Year Operating Stmt'!E14</f>
         <v>4035127</v>
       </c>
       <c r="F5" s="39">
+        <f>B5+'5-Year Operating Stmt'!C14+'5-Year Operating Stmt'!D14+'5-Year Operating Stmt'!E14+'5-Year Operating Stmt'!F14</f>
         <v>7149621</v>
       </c>
     </row>
@@ -4868,18 +4873,23 @@
         <v>335</v>
       </c>
       <c r="B9" s="31">
+        <f>SUM(B5:B8)</f>
         <v>74498</v>
       </c>
       <c r="C9" s="31">
+        <f>SUM(C5:C8)</f>
         <v>530168</v>
       </c>
       <c r="D9" s="31">
+        <f>SUM(D5:D8)</f>
         <v>1838758</v>
       </c>
       <c r="E9" s="31">
+        <f>SUM(E5:E8)</f>
         <v>4035127</v>
       </c>
       <c r="F9" s="31">
+        <f>SUM(F5:F8)</f>
         <v>7149621</v>
       </c>
     </row>
@@ -4918,18 +4928,23 @@
         <v>338</v>
       </c>
       <c r="B13" s="26">
+        <f>'Debt Schedule'!B13</f>
         <v>323655</v>
       </c>
       <c r="C13" s="26">
+        <f>'Debt Schedule'!C13</f>
         <v>295685</v>
       </c>
       <c r="D13" s="26">
+        <f>'Debt Schedule'!D13</f>
         <v>265989</v>
       </c>
       <c r="E13" s="26">
+        <f>'Debt Schedule'!E13</f>
         <v>234462</v>
       </c>
       <c r="F13" s="26">
+        <f>'Debt Schedule'!F13</f>
         <v>200991</v>
       </c>
     </row>
@@ -4938,18 +4953,23 @@
         <v>339</v>
       </c>
       <c r="B14" s="31">
+        <f>SUM(B12:B13)</f>
         <v>323655</v>
       </c>
       <c r="C14" s="31">
+        <f>SUM(C12:C13)</f>
         <v>295685</v>
       </c>
       <c r="D14" s="31">
+        <f>SUM(D12:D13)</f>
         <v>265989</v>
       </c>
       <c r="E14" s="31">
+        <f>SUM(E12:E13)</f>
         <v>234462</v>
       </c>
       <c r="F14" s="31">
+        <f>SUM(F12:F13)</f>
         <v>200991</v>
       </c>
     </row>
@@ -4968,18 +4988,23 @@
         <v>341</v>
       </c>
       <c r="B17" s="27">
+        <f>B9-B14</f>
         <v>-249157</v>
       </c>
       <c r="C17" s="27">
+        <f>C9-C14</f>
         <v>234484</v>
       </c>
       <c r="D17" s="27">
+        <f>D9-D14</f>
         <v>1572769</v>
       </c>
       <c r="E17" s="27">
+        <f>E9-E14</f>
         <v>3800665</v>
       </c>
       <c r="F17" s="27">
+        <f>F9-F14</f>
         <v>6948630</v>
       </c>
     </row>
@@ -4987,19 +5012,24 @@
       <c r="A19" s="3" t="s">
         <v>342</v>
       </c>
-      <c r="B19" s="40">
+      <c r="B19" s="40" t="str">
+        <f>B9-B14-B17</f>
         <v>0</v>
       </c>
       <c r="C19" s="41">
+        <f>C9-C14-C17</f>
         <v>-1</v>
       </c>
-      <c r="D19" s="40">
+      <c r="D19" s="40" t="str">
+        <f>D9-D14-D17</f>
         <v>0</v>
       </c>
-      <c r="E19" s="40">
+      <c r="E19" s="40" t="str">
+        <f>E9-E14-E17</f>
         <v>0</v>
       </c>
-      <c r="F19" s="40">
+      <c r="F19" s="40" t="str">
+        <f>F9-F14-F17</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>